<commit_message>
062425 - updated all skins data thru week 7.  week 8 is TBD
</commit_message>
<xml_diff>
--- a/public/results/2025/Week 6 Skins.xlsx
+++ b/public/results/2025/Week 6 Skins.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://amentumcms-my.sharepoint.com/personal/mark_hutter_amentumcms_com/Documents/DATA/Code/golf-league-site/public/results/2025/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{41632238-0933-4C67-8CBE-178E07F82065}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="28" documentId="8_{41632238-0933-4C67-8CBE-178E07F82065}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{F4CBDED5-D77B-4FF4-B005-081AA7281B45}"/>
   <bookViews>
-    <workbookView xWindow="6765" yWindow="1935" windowWidth="26730" windowHeight="18000" xr2:uid="{6533C28B-F533-48B1-90C7-82E9465E1322}"/>
+    <workbookView xWindow="43080" yWindow="3600" windowWidth="26730" windowHeight="18000" xr2:uid="{6533C28B-F533-48B1-90C7-82E9465E1322}"/>
   </bookViews>
   <sheets>
     <sheet name="Week 6 Skins" sheetId="1" r:id="rId1"/>
@@ -50,9 +50,6 @@
     <t>Hole</t>
   </si>
   <si>
-    <t>Hdcp</t>
-  </si>
-  <si>
     <t>PAR</t>
   </si>
   <si>
@@ -74,30 +71,12 @@
     <t>Skins ($30) $3.33/hole</t>
   </si>
   <si>
-    <t>Wise, Randy (15)</t>
-  </si>
-  <si>
     <t>Score</t>
   </si>
   <si>
     <t>Net</t>
   </si>
   <si>
-    <t>Ige, Shayne (22)</t>
-  </si>
-  <si>
-    <t>Morgan, Luke (10)</t>
-  </si>
-  <si>
-    <t>Hutter, Mark (8)</t>
-  </si>
-  <si>
-    <t>Miller, Ryan (8)</t>
-  </si>
-  <si>
-    <t>Walters, Kevin (17)</t>
-  </si>
-  <si>
     <t>Wise (1)</t>
   </si>
   <si>
@@ -114,6 +93,27 @@
   </si>
   <si>
     <t>Miller (1)</t>
+  </si>
+  <si>
+    <t>HDCP</t>
+  </si>
+  <si>
+    <t>Randy W</t>
+  </si>
+  <si>
+    <t>Shayne I</t>
+  </si>
+  <si>
+    <t>Luke M</t>
+  </si>
+  <si>
+    <t>Mark H</t>
+  </si>
+  <si>
+    <t>Ryan M</t>
+  </si>
+  <si>
+    <t>Kevin W</t>
   </si>
 </sst>
 </file>
@@ -123,7 +123,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0.00"/>
   </numFmts>
-  <fonts count="7" x14ac:knownFonts="1">
+  <fonts count="11" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -170,6 +170,32 @@
       <name val="Arial"/>
       <family val="2"/>
     </font>
+    <font>
+      <sz val="10"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="9"/>
+      <color theme="1"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="9"/>
+      <color theme="1"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="9"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
   <fills count="6">
     <fill>
@@ -335,19 +361,6 @@
       <diagonal/>
     </border>
     <border>
-      <left style="thin">
-        <color rgb="FFAEABAB"/>
-      </left>
-      <right/>
-      <top style="thin">
-        <color rgb="FFAEABAB"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FFAEABAB"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
       <left style="medium">
         <color indexed="64"/>
       </left>
@@ -477,19 +490,6 @@
       <left style="medium">
         <color indexed="64"/>
       </left>
-      <right/>
-      <top style="medium">
-        <color indexed="64"/>
-      </top>
-      <bottom style="medium">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="medium">
-        <color indexed="64"/>
-      </left>
       <right style="thin">
         <color rgb="FFAEABAB"/>
       </right>
@@ -524,17 +524,6 @@
       <diagonal/>
     </border>
     <border>
-      <left style="thin">
-        <color rgb="FFAEABAB"/>
-      </left>
-      <right/>
-      <top/>
-      <bottom style="thin">
-        <color rgb="FFAEABAB"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
       <left style="medium">
         <color indexed="64"/>
       </left>
@@ -556,6 +545,41 @@
       </right>
       <top/>
       <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FFAEABAB"/>
+      </left>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FFAEABAB"/>
+      </left>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
       <diagonal/>
     </border>
   </borders>
@@ -563,7 +587,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="45">
+  <cellXfs count="52">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -574,16 +598,10 @@
     <xf numFmtId="0" fontId="3" fillId="3" borderId="9" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="10" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="12" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="4" borderId="13" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="4" borderId="14" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="4" borderId="15" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -595,31 +613,31 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="5" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="11" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="10" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="16" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="15" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="16" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="17" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="18" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="12" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="13" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="13" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="13" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="14" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="5" borderId="14" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="15" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="19" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="18" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1"/>
@@ -629,31 +647,22 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="21" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="20" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="22" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="22" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="23" xfId="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="24" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="25" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="26" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="23" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="27" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="24" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="6" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="164" fontId="3" fillId="0" borderId="23" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="3" fillId="0" borderId="21" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="164" fontId="3" fillId="0" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -665,10 +674,10 @@
     <xf numFmtId="164" fontId="4" fillId="0" borderId="7" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="12" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="11" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="20" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="19" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
     <xf numFmtId="164" fontId="1" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyAlignment="1">
@@ -677,24 +686,56 @@
     <xf numFmtId="164" fontId="3" fillId="0" borderId="2" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="164" fontId="3" fillId="0" borderId="26" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="3" fillId="0" borderId="23" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="164" fontId="3" fillId="0" borderId="27" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="3" fillId="0" borderId="24" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
     <xf numFmtId="164" fontId="3" fillId="0" borderId="6" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="164" fontId="3" fillId="0" borderId="11" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="3" fillId="0" borderId="10" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="164" fontId="3" fillId="0" borderId="19" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="3" fillId="0" borderId="18" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
     <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="25" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="26" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="180"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="27" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="180"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="4" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="16" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="13" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="8" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="9" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1033,79 +1074,83 @@
   <dimension ref="A1:O25"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="3" max="12" width="10.7109375" customWidth="1"/>
-    <col min="13" max="13" width="6.85546875" style="22" customWidth="1"/>
-    <col min="14" max="15" width="7" style="22" customWidth="1"/>
+    <col min="1" max="1" width="10.28515625" customWidth="1"/>
+    <col min="2" max="2" width="9" customWidth="1"/>
+    <col min="3" max="11" width="8.7109375" customWidth="1"/>
+    <col min="12" max="12" width="3.85546875" customWidth="1"/>
+    <col min="13" max="13" width="5.85546875" style="20" customWidth="1"/>
+    <col min="14" max="14" width="6.85546875" style="20" customWidth="1"/>
+    <col min="15" max="15" width="6.42578125" style="20" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:15" ht="30.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="23" t="s">
-        <v>11</v>
-      </c>
-      <c r="B1" s="25"/>
-      <c r="C1" s="25"/>
-      <c r="D1" s="25"/>
-      <c r="E1" s="25"/>
-      <c r="F1" s="25"/>
-      <c r="G1" s="25"/>
-      <c r="H1" s="25"/>
-      <c r="I1" s="25"/>
-      <c r="J1" s="25"/>
-      <c r="K1" s="25"/>
-      <c r="L1" s="25"/>
+      <c r="A1" s="40" t="s">
+        <v>10</v>
+      </c>
+      <c r="B1" s="41"/>
+      <c r="C1" s="41"/>
+      <c r="D1" s="41"/>
+      <c r="E1" s="41"/>
+      <c r="F1" s="41"/>
+      <c r="G1" s="41"/>
+      <c r="H1" s="41"/>
+      <c r="I1" s="41"/>
+      <c r="J1" s="41"/>
+      <c r="K1" s="41"/>
+      <c r="L1" s="41"/>
       <c r="M1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="N1" s="31"/>
-      <c r="O1" s="38" t="s">
+      <c r="N1" s="26"/>
+      <c r="O1" s="33" t="s">
         <v>1</v>
       </c>
     </row>
     <row r="2" spans="1:15" ht="18.75" x14ac:dyDescent="0.25">
-      <c r="A2" s="24" t="s">
-        <v>2</v>
-      </c>
-      <c r="B2" s="26" t="s">
-        <v>3</v>
-      </c>
-      <c r="C2" s="26">
-        <v>1</v>
-      </c>
-      <c r="D2" s="26">
-        <v>2</v>
-      </c>
-      <c r="E2" s="26">
-        <v>3</v>
-      </c>
-      <c r="F2" s="26">
-        <v>4</v>
-      </c>
-      <c r="G2" s="26">
-        <v>5</v>
-      </c>
-      <c r="H2" s="26">
-        <v>6</v>
-      </c>
-      <c r="I2" s="26">
+      <c r="A2" s="21" t="s">
+        <v>2</v>
+      </c>
+      <c r="B2" s="22" t="s">
+        <v>3</v>
+      </c>
+      <c r="C2" s="22">
+        <v>1</v>
+      </c>
+      <c r="D2" s="22">
+        <v>2</v>
+      </c>
+      <c r="E2" s="22">
+        <v>3</v>
+      </c>
+      <c r="F2" s="22">
+        <v>4</v>
+      </c>
+      <c r="G2" s="22">
+        <v>5</v>
+      </c>
+      <c r="H2" s="22">
+        <v>6</v>
+      </c>
+      <c r="I2" s="22">
         <v>7</v>
       </c>
-      <c r="J2" s="26">
+      <c r="J2" s="22">
         <v>8</v>
       </c>
-      <c r="K2" s="26">
+      <c r="K2" s="22">
         <v>9</v>
       </c>
-      <c r="L2" s="27" t="s">
-        <v>4</v>
-      </c>
-      <c r="M2" s="28"/>
-      <c r="N2" s="32"/>
-      <c r="O2" s="39"/>
+      <c r="L2" s="42" t="s">
+        <v>19</v>
+      </c>
+      <c r="M2" s="23"/>
+      <c r="N2" s="27"/>
+      <c r="O2" s="34"/>
     </row>
     <row r="3" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A3" s="2"/>
       <c r="B3" s="3" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="C3" s="3">
         <v>4</v>
@@ -1134,914 +1179,916 @@
       <c r="K3" s="3">
         <v>5</v>
       </c>
-      <c r="L3" s="4"/>
-      <c r="M3" s="29"/>
-      <c r="N3" s="33"/>
-      <c r="O3" s="40"/>
+      <c r="L3" s="42"/>
+      <c r="M3" s="24"/>
+      <c r="N3" s="28"/>
+      <c r="O3" s="35"/>
     </row>
     <row r="4" spans="1:15" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A4" s="5"/>
-      <c r="B4" s="6" t="s">
-        <v>6</v>
-      </c>
-      <c r="C4" s="6">
-        <v>4</v>
-      </c>
-      <c r="D4" s="6">
-        <v>1</v>
-      </c>
-      <c r="E4" s="6">
-        <v>3</v>
-      </c>
-      <c r="F4" s="6">
+      <c r="A4" s="4"/>
+      <c r="B4" s="5" t="s">
+        <v>5</v>
+      </c>
+      <c r="C4" s="5">
+        <v>4</v>
+      </c>
+      <c r="D4" s="5">
+        <v>1</v>
+      </c>
+      <c r="E4" s="5">
+        <v>3</v>
+      </c>
+      <c r="F4" s="5">
         <v>9</v>
       </c>
-      <c r="G4" s="6">
-        <v>5</v>
-      </c>
-      <c r="H4" s="6">
+      <c r="G4" s="5">
+        <v>5</v>
+      </c>
+      <c r="H4" s="5">
         <v>7</v>
       </c>
-      <c r="I4" s="6">
+      <c r="I4" s="5">
         <v>8</v>
       </c>
-      <c r="J4" s="6">
-        <v>6</v>
-      </c>
-      <c r="K4" s="6">
-        <v>2</v>
-      </c>
-      <c r="L4" s="7"/>
-      <c r="M4" s="29"/>
-      <c r="N4" s="33"/>
-      <c r="O4" s="40"/>
+      <c r="J4" s="5">
+        <v>6</v>
+      </c>
+      <c r="K4" s="5">
+        <v>2</v>
+      </c>
+      <c r="L4" s="43"/>
+      <c r="M4" s="24"/>
+      <c r="N4" s="28"/>
+      <c r="O4" s="35"/>
     </row>
     <row r="5" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A5" s="8" t="s">
-        <v>12</v>
-      </c>
-      <c r="B5" s="9" t="s">
-        <v>13</v>
-      </c>
-      <c r="C5" s="9">
-        <v>6</v>
-      </c>
-      <c r="D5" s="9">
-        <v>5</v>
-      </c>
-      <c r="E5" s="9">
-        <v>4</v>
-      </c>
-      <c r="F5" s="9">
-        <v>3</v>
-      </c>
-      <c r="G5" s="9">
+      <c r="A5" s="6" t="s">
+        <v>20</v>
+      </c>
+      <c r="B5" s="44" t="s">
+        <v>11</v>
+      </c>
+      <c r="C5" s="7">
+        <v>6</v>
+      </c>
+      <c r="D5" s="7">
+        <v>5</v>
+      </c>
+      <c r="E5" s="7">
+        <v>4</v>
+      </c>
+      <c r="F5" s="7">
+        <v>3</v>
+      </c>
+      <c r="G5" s="7">
         <v>7</v>
       </c>
-      <c r="H5" s="9">
-        <v>6</v>
-      </c>
-      <c r="I5" s="9">
-        <v>4</v>
-      </c>
-      <c r="J5" s="9">
-        <v>6</v>
-      </c>
-      <c r="K5" s="9">
-        <v>5</v>
-      </c>
-      <c r="L5" s="10"/>
-      <c r="M5" s="30"/>
-      <c r="N5" s="34"/>
-      <c r="O5" s="41"/>
+      <c r="H5" s="7">
+        <v>6</v>
+      </c>
+      <c r="I5" s="7">
+        <v>4</v>
+      </c>
+      <c r="J5" s="7">
+        <v>6</v>
+      </c>
+      <c r="K5" s="7">
+        <v>5</v>
+      </c>
+      <c r="L5" s="8"/>
+      <c r="M5" s="25"/>
+      <c r="N5" s="29"/>
+      <c r="O5" s="36"/>
     </row>
     <row r="6" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A6" s="12"/>
-      <c r="B6" s="13" t="s">
-        <v>7</v>
-      </c>
-      <c r="C6" s="13">
-        <v>2</v>
-      </c>
-      <c r="D6" s="13">
-        <v>2</v>
-      </c>
-      <c r="E6" s="13">
-        <v>2</v>
-      </c>
-      <c r="F6" s="13">
-        <v>1</v>
-      </c>
-      <c r="G6" s="13">
-        <v>2</v>
-      </c>
-      <c r="H6" s="13">
-        <v>1</v>
-      </c>
-      <c r="I6" s="13">
-        <v>1</v>
-      </c>
-      <c r="J6" s="13">
-        <v>2</v>
-      </c>
-      <c r="K6" s="13">
-        <v>2</v>
-      </c>
-      <c r="L6" s="14">
+      <c r="A6" s="10"/>
+      <c r="B6" s="45" t="s">
+        <v>6</v>
+      </c>
+      <c r="C6" s="11">
+        <v>2</v>
+      </c>
+      <c r="D6" s="11">
+        <v>2</v>
+      </c>
+      <c r="E6" s="11">
+        <v>2</v>
+      </c>
+      <c r="F6" s="11">
+        <v>1</v>
+      </c>
+      <c r="G6" s="11">
+        <v>2</v>
+      </c>
+      <c r="H6" s="11">
+        <v>1</v>
+      </c>
+      <c r="I6" s="11">
+        <v>1</v>
+      </c>
+      <c r="J6" s="11">
+        <v>2</v>
+      </c>
+      <c r="K6" s="11">
+        <v>2</v>
+      </c>
+      <c r="L6" s="12">
         <f>SUM(C6:K6)</f>
         <v>15</v>
       </c>
-      <c r="M6" s="11"/>
-      <c r="N6" s="35"/>
-      <c r="O6" s="42"/>
+      <c r="M6" s="9"/>
+      <c r="N6" s="30"/>
+      <c r="O6" s="37"/>
     </row>
     <row r="7" spans="1:15" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A7" s="15"/>
-      <c r="B7" s="16" t="s">
-        <v>14</v>
-      </c>
-      <c r="C7" s="16">
+      <c r="A7" s="13"/>
+      <c r="B7" s="46" t="s">
+        <v>12</v>
+      </c>
+      <c r="C7" s="14">
         <f>C5-C6</f>
         <v>4</v>
       </c>
-      <c r="D7" s="17">
+      <c r="D7" s="15">
         <f t="shared" ref="D7:K7" si="0">D5-D6</f>
         <v>3</v>
       </c>
-      <c r="E7" s="17">
+      <c r="E7" s="15">
         <f t="shared" si="0"/>
         <v>2</v>
       </c>
-      <c r="F7" s="17">
+      <c r="F7" s="15">
         <f t="shared" si="0"/>
         <v>2</v>
       </c>
-      <c r="G7" s="16">
+      <c r="G7" s="14">
         <f t="shared" si="0"/>
         <v>5</v>
       </c>
-      <c r="H7" s="16">
+      <c r="H7" s="14">
         <f t="shared" si="0"/>
         <v>5</v>
       </c>
-      <c r="I7" s="16">
+      <c r="I7" s="14">
         <f t="shared" si="0"/>
         <v>3</v>
       </c>
-      <c r="J7" s="16">
+      <c r="J7" s="14">
         <f t="shared" si="0"/>
         <v>4</v>
       </c>
-      <c r="K7" s="17">
+      <c r="K7" s="15">
         <f t="shared" si="0"/>
         <v>3</v>
       </c>
-      <c r="L7" s="18"/>
-      <c r="M7" s="11">
+      <c r="L7" s="16"/>
+      <c r="M7" s="9">
         <v>2.5</v>
       </c>
-      <c r="N7" s="35">
+      <c r="N7" s="30">
         <v>8.33</v>
       </c>
-      <c r="O7" s="42">
+      <c r="O7" s="37">
         <v>8</v>
       </c>
     </row>
     <row r="8" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A8" s="8" t="s">
-        <v>15</v>
-      </c>
-      <c r="B8" s="9" t="s">
-        <v>13</v>
-      </c>
-      <c r="C8" s="9">
-        <v>5</v>
-      </c>
-      <c r="D8" s="9">
+      <c r="A8" s="6" t="s">
+        <v>21</v>
+      </c>
+      <c r="B8" s="44" t="s">
+        <v>11</v>
+      </c>
+      <c r="C8" s="7">
+        <v>5</v>
+      </c>
+      <c r="D8" s="7">
         <v>9</v>
       </c>
-      <c r="E8" s="9">
+      <c r="E8" s="7">
         <v>7</v>
       </c>
-      <c r="F8" s="9">
-        <v>4</v>
-      </c>
-      <c r="G8" s="9">
+      <c r="F8" s="7">
+        <v>4</v>
+      </c>
+      <c r="G8" s="7">
         <v>8</v>
       </c>
-      <c r="H8" s="9">
-        <v>6</v>
-      </c>
-      <c r="I8" s="9">
-        <v>6</v>
-      </c>
-      <c r="J8" s="9">
-        <v>5</v>
-      </c>
-      <c r="K8" s="9">
-        <v>6</v>
-      </c>
-      <c r="L8" s="10"/>
-      <c r="M8" s="11"/>
-      <c r="N8" s="35"/>
-      <c r="O8" s="42"/>
+      <c r="H8" s="7">
+        <v>6</v>
+      </c>
+      <c r="I8" s="7">
+        <v>6</v>
+      </c>
+      <c r="J8" s="7">
+        <v>5</v>
+      </c>
+      <c r="K8" s="7">
+        <v>6</v>
+      </c>
+      <c r="L8" s="8"/>
+      <c r="M8" s="9"/>
+      <c r="N8" s="30"/>
+      <c r="O8" s="37"/>
     </row>
     <row r="9" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A9" s="12"/>
-      <c r="B9" s="13" t="s">
-        <v>7</v>
-      </c>
-      <c r="C9" s="13">
-        <v>3</v>
-      </c>
-      <c r="D9" s="13">
-        <v>3</v>
-      </c>
-      <c r="E9" s="13">
-        <v>3</v>
-      </c>
-      <c r="F9" s="13">
-        <v>2</v>
-      </c>
-      <c r="G9" s="13">
-        <v>2</v>
-      </c>
-      <c r="H9" s="13">
-        <v>2</v>
-      </c>
-      <c r="I9" s="13">
-        <v>2</v>
-      </c>
-      <c r="J9" s="13">
-        <v>2</v>
-      </c>
-      <c r="K9" s="13">
-        <v>3</v>
-      </c>
-      <c r="L9" s="14">
+      <c r="A9" s="10"/>
+      <c r="B9" s="45" t="s">
+        <v>6</v>
+      </c>
+      <c r="C9" s="11">
+        <v>3</v>
+      </c>
+      <c r="D9" s="11">
+        <v>3</v>
+      </c>
+      <c r="E9" s="11">
+        <v>3</v>
+      </c>
+      <c r="F9" s="11">
+        <v>2</v>
+      </c>
+      <c r="G9" s="11">
+        <v>2</v>
+      </c>
+      <c r="H9" s="11">
+        <v>2</v>
+      </c>
+      <c r="I9" s="11">
+        <v>2</v>
+      </c>
+      <c r="J9" s="11">
+        <v>2</v>
+      </c>
+      <c r="K9" s="11">
+        <v>3</v>
+      </c>
+      <c r="L9" s="12">
         <f>SUM(C9:K9)</f>
         <v>22</v>
       </c>
-      <c r="M9" s="11"/>
-      <c r="N9" s="35"/>
-      <c r="O9" s="42"/>
+      <c r="M9" s="9"/>
+      <c r="N9" s="30"/>
+      <c r="O9" s="37"/>
     </row>
     <row r="10" spans="1:15" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A10" s="15"/>
-      <c r="B10" s="16" t="s">
-        <v>14</v>
-      </c>
-      <c r="C10" s="17">
+      <c r="A10" s="13"/>
+      <c r="B10" s="46" t="s">
+        <v>12</v>
+      </c>
+      <c r="C10" s="15">
         <f>C8-C9</f>
         <v>2</v>
       </c>
-      <c r="D10" s="16">
+      <c r="D10" s="14">
         <f t="shared" ref="D10:K10" si="1">D8-D9</f>
         <v>6</v>
       </c>
-      <c r="E10" s="16">
+      <c r="E10" s="14">
         <f t="shared" si="1"/>
         <v>4</v>
       </c>
-      <c r="F10" s="17">
+      <c r="F10" s="15">
         <f t="shared" si="1"/>
         <v>2</v>
       </c>
-      <c r="G10" s="16">
+      <c r="G10" s="14">
         <f t="shared" si="1"/>
         <v>6</v>
       </c>
-      <c r="H10" s="16">
+      <c r="H10" s="14">
         <f t="shared" si="1"/>
         <v>4</v>
       </c>
-      <c r="I10" s="16">
+      <c r="I10" s="14">
         <f t="shared" si="1"/>
         <v>4</v>
       </c>
-      <c r="J10" s="17">
+      <c r="J10" s="15">
         <f t="shared" si="1"/>
         <v>3</v>
       </c>
-      <c r="K10" s="17">
+      <c r="K10" s="15">
         <f t="shared" si="1"/>
         <v>3</v>
       </c>
-      <c r="L10" s="18"/>
-      <c r="M10" s="11">
+      <c r="L10" s="16"/>
+      <c r="M10" s="9">
         <v>2.5</v>
       </c>
-      <c r="N10" s="35">
+      <c r="N10" s="30">
         <v>8.33</v>
       </c>
-      <c r="O10" s="42">
+      <c r="O10" s="37">
         <v>8</v>
       </c>
     </row>
     <row r="11" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A11" s="8" t="s">
-        <v>16</v>
-      </c>
-      <c r="B11" s="9" t="s">
-        <v>13</v>
-      </c>
-      <c r="C11" s="9">
-        <v>4</v>
-      </c>
-      <c r="D11" s="9">
+      <c r="A11" s="6" t="s">
+        <v>22</v>
+      </c>
+      <c r="B11" s="44" t="s">
+        <v>11</v>
+      </c>
+      <c r="C11" s="7">
+        <v>4</v>
+      </c>
+      <c r="D11" s="7">
         <v>7</v>
       </c>
-      <c r="E11" s="9">
-        <v>6</v>
-      </c>
-      <c r="F11" s="9">
-        <v>4</v>
-      </c>
-      <c r="G11" s="9">
-        <v>4</v>
-      </c>
-      <c r="H11" s="9">
-        <v>6</v>
-      </c>
-      <c r="I11" s="9">
-        <v>3</v>
-      </c>
-      <c r="J11" s="9">
-        <v>6</v>
-      </c>
-      <c r="K11" s="9">
-        <v>6</v>
-      </c>
-      <c r="L11" s="10">
+      <c r="E11" s="7">
+        <v>6</v>
+      </c>
+      <c r="F11" s="7">
+        <v>4</v>
+      </c>
+      <c r="G11" s="7">
+        <v>4</v>
+      </c>
+      <c r="H11" s="7">
+        <v>6</v>
+      </c>
+      <c r="I11" s="7">
+        <v>3</v>
+      </c>
+      <c r="J11" s="7">
+        <v>6</v>
+      </c>
+      <c r="K11" s="7">
+        <v>6</v>
+      </c>
+      <c r="L11" s="8">
         <v>10</v>
       </c>
-      <c r="M11" s="11"/>
-      <c r="N11" s="35"/>
-      <c r="O11" s="42"/>
+      <c r="M11" s="9"/>
+      <c r="N11" s="30"/>
+      <c r="O11" s="37"/>
     </row>
     <row r="12" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A12" s="12"/>
-      <c r="B12" s="13" t="s">
-        <v>7</v>
-      </c>
-      <c r="C12" s="13">
-        <v>1</v>
-      </c>
-      <c r="D12" s="13">
-        <v>2</v>
-      </c>
-      <c r="E12" s="13">
-        <v>1</v>
-      </c>
-      <c r="F12" s="13">
-        <v>1</v>
-      </c>
-      <c r="G12" s="13">
-        <v>1</v>
-      </c>
-      <c r="H12" s="13">
-        <v>1</v>
-      </c>
-      <c r="I12" s="13">
-        <v>1</v>
-      </c>
-      <c r="J12" s="13">
-        <v>1</v>
-      </c>
-      <c r="K12" s="13">
-        <v>1</v>
-      </c>
-      <c r="L12" s="14"/>
-      <c r="M12" s="11"/>
-      <c r="N12" s="35"/>
-      <c r="O12" s="42"/>
+      <c r="A12" s="10"/>
+      <c r="B12" s="45" t="s">
+        <v>6</v>
+      </c>
+      <c r="C12" s="11">
+        <v>1</v>
+      </c>
+      <c r="D12" s="11">
+        <v>2</v>
+      </c>
+      <c r="E12" s="11">
+        <v>1</v>
+      </c>
+      <c r="F12" s="11">
+        <v>1</v>
+      </c>
+      <c r="G12" s="11">
+        <v>1</v>
+      </c>
+      <c r="H12" s="11">
+        <v>1</v>
+      </c>
+      <c r="I12" s="11">
+        <v>1</v>
+      </c>
+      <c r="J12" s="11">
+        <v>1</v>
+      </c>
+      <c r="K12" s="11">
+        <v>1</v>
+      </c>
+      <c r="L12" s="12"/>
+      <c r="M12" s="9"/>
+      <c r="N12" s="30"/>
+      <c r="O12" s="37"/>
     </row>
     <row r="13" spans="1:15" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A13" s="15"/>
-      <c r="B13" s="16" t="s">
-        <v>14</v>
-      </c>
-      <c r="C13" s="16">
+      <c r="A13" s="13"/>
+      <c r="B13" s="46" t="s">
+        <v>12</v>
+      </c>
+      <c r="C13" s="14">
         <f>C11-C12</f>
         <v>3</v>
       </c>
-      <c r="D13" s="16">
+      <c r="D13" s="14">
         <f t="shared" ref="D13:K13" si="2">D11-D12</f>
         <v>5</v>
       </c>
-      <c r="E13" s="16">
+      <c r="E13" s="14">
         <f t="shared" si="2"/>
         <v>5</v>
       </c>
-      <c r="F13" s="16">
+      <c r="F13" s="14">
         <f t="shared" si="2"/>
         <v>3</v>
       </c>
-      <c r="G13" s="17">
+      <c r="G13" s="15">
         <f t="shared" si="2"/>
         <v>3</v>
       </c>
-      <c r="H13" s="16">
+      <c r="H13" s="14">
         <f t="shared" si="2"/>
         <v>5</v>
       </c>
-      <c r="I13" s="17">
+      <c r="I13" s="15">
         <f t="shared" si="2"/>
         <v>2</v>
       </c>
-      <c r="J13" s="16">
+      <c r="J13" s="14">
         <f t="shared" si="2"/>
         <v>5</v>
       </c>
-      <c r="K13" s="16">
+      <c r="K13" s="14">
         <f t="shared" si="2"/>
         <v>5</v>
       </c>
-      <c r="L13" s="18"/>
-      <c r="M13" s="11">
-        <v>1</v>
-      </c>
-      <c r="N13" s="35">
+      <c r="L13" s="16"/>
+      <c r="M13" s="9">
+        <v>1</v>
+      </c>
+      <c r="N13" s="30">
         <v>3.33</v>
       </c>
-      <c r="O13" s="42">
+      <c r="O13" s="37">
         <v>3</v>
       </c>
     </row>
     <row r="14" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A14" s="8" t="s">
-        <v>17</v>
-      </c>
-      <c r="B14" s="9" t="s">
-        <v>13</v>
-      </c>
-      <c r="C14" s="9">
-        <v>4</v>
-      </c>
-      <c r="D14" s="9">
-        <v>5</v>
-      </c>
-      <c r="E14" s="9">
-        <v>6</v>
-      </c>
-      <c r="F14" s="9">
-        <v>3</v>
-      </c>
-      <c r="G14" s="9">
-        <v>6</v>
-      </c>
-      <c r="H14" s="9">
-        <v>4</v>
-      </c>
-      <c r="I14" s="9">
-        <v>4</v>
-      </c>
-      <c r="J14" s="9">
-        <v>5</v>
-      </c>
-      <c r="K14" s="9">
-        <v>4</v>
-      </c>
-      <c r="L14" s="10"/>
-      <c r="M14" s="11"/>
-      <c r="N14" s="35"/>
-      <c r="O14" s="42"/>
+      <c r="A14" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="B14" s="44" t="s">
+        <v>11</v>
+      </c>
+      <c r="C14" s="7">
+        <v>4</v>
+      </c>
+      <c r="D14" s="7">
+        <v>5</v>
+      </c>
+      <c r="E14" s="7">
+        <v>6</v>
+      </c>
+      <c r="F14" s="7">
+        <v>3</v>
+      </c>
+      <c r="G14" s="7">
+        <v>6</v>
+      </c>
+      <c r="H14" s="7">
+        <v>4</v>
+      </c>
+      <c r="I14" s="7">
+        <v>4</v>
+      </c>
+      <c r="J14" s="7">
+        <v>5</v>
+      </c>
+      <c r="K14" s="7">
+        <v>4</v>
+      </c>
+      <c r="L14" s="8"/>
+      <c r="M14" s="9"/>
+      <c r="N14" s="30"/>
+      <c r="O14" s="37"/>
     </row>
     <row r="15" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A15" s="12"/>
-      <c r="B15" s="13" t="s">
-        <v>7</v>
-      </c>
-      <c r="C15" s="13">
-        <v>1</v>
-      </c>
-      <c r="D15" s="13">
-        <v>1</v>
-      </c>
-      <c r="E15" s="13">
-        <v>1</v>
-      </c>
-      <c r="F15" s="13">
+      <c r="A15" s="10"/>
+      <c r="B15" s="45" t="s">
+        <v>6</v>
+      </c>
+      <c r="C15" s="11">
+        <v>1</v>
+      </c>
+      <c r="D15" s="11">
+        <v>1</v>
+      </c>
+      <c r="E15" s="11">
+        <v>1</v>
+      </c>
+      <c r="F15" s="11">
         <v>0</v>
       </c>
-      <c r="G15" s="13">
-        <v>1</v>
-      </c>
-      <c r="H15" s="13">
-        <v>1</v>
-      </c>
-      <c r="I15" s="13">
-        <v>1</v>
-      </c>
-      <c r="J15" s="13">
-        <v>1</v>
-      </c>
-      <c r="K15" s="13">
-        <v>1</v>
-      </c>
-      <c r="L15" s="14">
+      <c r="G15" s="11">
+        <v>1</v>
+      </c>
+      <c r="H15" s="11">
+        <v>1</v>
+      </c>
+      <c r="I15" s="11">
+        <v>1</v>
+      </c>
+      <c r="J15" s="11">
+        <v>1</v>
+      </c>
+      <c r="K15" s="11">
+        <v>1</v>
+      </c>
+      <c r="L15" s="12">
         <f>SUM(C15:K15)</f>
         <v>8</v>
       </c>
-      <c r="M15" s="11"/>
-      <c r="N15" s="35"/>
-      <c r="O15" s="42"/>
+      <c r="M15" s="9"/>
+      <c r="N15" s="30"/>
+      <c r="O15" s="37"/>
     </row>
     <row r="16" spans="1:15" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A16" s="15"/>
-      <c r="B16" s="16" t="s">
-        <v>14</v>
-      </c>
-      <c r="C16" s="16">
+      <c r="A16" s="13"/>
+      <c r="B16" s="46" t="s">
+        <v>12</v>
+      </c>
+      <c r="C16" s="14">
         <f>C14-C15</f>
         <v>3</v>
       </c>
-      <c r="D16" s="16">
+      <c r="D16" s="14">
         <f t="shared" ref="D16:K16" si="3">D14-D15</f>
         <v>4</v>
       </c>
-      <c r="E16" s="16">
+      <c r="E16" s="14">
         <f t="shared" si="3"/>
         <v>5</v>
       </c>
-      <c r="F16" s="16">
+      <c r="F16" s="14">
         <f t="shared" si="3"/>
         <v>3</v>
       </c>
-      <c r="G16" s="16">
+      <c r="G16" s="14">
         <f t="shared" si="3"/>
         <v>5</v>
       </c>
-      <c r="H16" s="17">
+      <c r="H16" s="15">
         <f t="shared" si="3"/>
         <v>3</v>
       </c>
-      <c r="I16" s="16">
+      <c r="I16" s="14">
         <f t="shared" si="3"/>
         <v>3</v>
       </c>
-      <c r="J16" s="16">
+      <c r="J16" s="14">
         <f t="shared" si="3"/>
         <v>4</v>
       </c>
-      <c r="K16" s="17">
+      <c r="K16" s="15">
         <f t="shared" si="3"/>
         <v>3</v>
       </c>
-      <c r="L16" s="18"/>
-      <c r="M16" s="11">
-        <v>1</v>
-      </c>
-      <c r="N16" s="35">
+      <c r="L16" s="16"/>
+      <c r="M16" s="9">
+        <v>1</v>
+      </c>
+      <c r="N16" s="30">
         <v>3.33</v>
       </c>
-      <c r="O16" s="42">
+      <c r="O16" s="37">
         <v>3</v>
       </c>
     </row>
     <row r="17" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A17" s="8" t="s">
-        <v>18</v>
-      </c>
-      <c r="B17" s="9" t="s">
-        <v>13</v>
-      </c>
-      <c r="C17" s="9">
-        <v>5</v>
-      </c>
-      <c r="D17" s="9">
-        <v>5</v>
-      </c>
-      <c r="E17" s="9">
+      <c r="A17" s="6" t="s">
+        <v>24</v>
+      </c>
+      <c r="B17" s="44" t="s">
+        <v>11</v>
+      </c>
+      <c r="C17" s="7">
+        <v>5</v>
+      </c>
+      <c r="D17" s="7">
+        <v>5</v>
+      </c>
+      <c r="E17" s="7">
         <v>7</v>
       </c>
-      <c r="F17" s="9">
-        <v>3</v>
-      </c>
-      <c r="G17" s="9">
-        <v>5</v>
-      </c>
-      <c r="H17" s="9">
-        <v>6</v>
-      </c>
-      <c r="I17" s="9">
-        <v>3</v>
-      </c>
-      <c r="J17" s="9">
-        <v>4</v>
-      </c>
-      <c r="K17" s="9">
-        <v>4</v>
-      </c>
-      <c r="L17" s="10"/>
-      <c r="M17" s="11"/>
-      <c r="N17" s="35"/>
-      <c r="O17" s="42"/>
+      <c r="F17" s="7">
+        <v>3</v>
+      </c>
+      <c r="G17" s="7">
+        <v>5</v>
+      </c>
+      <c r="H17" s="7">
+        <v>6</v>
+      </c>
+      <c r="I17" s="7">
+        <v>3</v>
+      </c>
+      <c r="J17" s="7">
+        <v>4</v>
+      </c>
+      <c r="K17" s="7">
+        <v>4</v>
+      </c>
+      <c r="L17" s="8"/>
+      <c r="M17" s="9"/>
+      <c r="N17" s="30"/>
+      <c r="O17" s="37"/>
     </row>
     <row r="18" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A18" s="12"/>
-      <c r="B18" s="13" t="s">
-        <v>7</v>
-      </c>
-      <c r="C18" s="13">
-        <v>1</v>
-      </c>
-      <c r="D18" s="13">
-        <v>1</v>
-      </c>
-      <c r="E18" s="13">
-        <v>1</v>
-      </c>
-      <c r="F18" s="13">
+      <c r="A18" s="10"/>
+      <c r="B18" s="45" t="s">
+        <v>6</v>
+      </c>
+      <c r="C18" s="11">
+        <v>1</v>
+      </c>
+      <c r="D18" s="11">
+        <v>1</v>
+      </c>
+      <c r="E18" s="11">
+        <v>1</v>
+      </c>
+      <c r="F18" s="11">
         <v>0</v>
       </c>
-      <c r="G18" s="13">
-        <v>1</v>
-      </c>
-      <c r="H18" s="13">
-        <v>1</v>
-      </c>
-      <c r="I18" s="13">
-        <v>1</v>
-      </c>
-      <c r="J18" s="13">
-        <v>1</v>
-      </c>
-      <c r="K18" s="13">
-        <v>1</v>
-      </c>
-      <c r="L18" s="14">
+      <c r="G18" s="11">
+        <v>1</v>
+      </c>
+      <c r="H18" s="11">
+        <v>1</v>
+      </c>
+      <c r="I18" s="11">
+        <v>1</v>
+      </c>
+      <c r="J18" s="11">
+        <v>1</v>
+      </c>
+      <c r="K18" s="11">
+        <v>1</v>
+      </c>
+      <c r="L18" s="12">
         <f>SUM(C18:K18)</f>
         <v>8</v>
       </c>
-      <c r="M18" s="11"/>
-      <c r="N18" s="35"/>
-      <c r="O18" s="42"/>
+      <c r="M18" s="9"/>
+      <c r="N18" s="30"/>
+      <c r="O18" s="37"/>
     </row>
     <row r="19" spans="1:15" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A19" s="15"/>
-      <c r="B19" s="16" t="s">
-        <v>14</v>
-      </c>
-      <c r="C19" s="16">
+      <c r="A19" s="13"/>
+      <c r="B19" s="46" t="s">
+        <v>12</v>
+      </c>
+      <c r="C19" s="14">
         <f>C17-C18</f>
         <v>4</v>
       </c>
-      <c r="D19" s="16">
+      <c r="D19" s="14">
         <f t="shared" ref="D19:K19" si="4">D17-D18</f>
         <v>4</v>
       </c>
-      <c r="E19" s="16">
+      <c r="E19" s="14">
         <f t="shared" si="4"/>
         <v>6</v>
       </c>
-      <c r="F19" s="16">
+      <c r="F19" s="14">
         <f t="shared" si="4"/>
         <v>3</v>
       </c>
-      <c r="G19" s="16">
+      <c r="G19" s="14">
         <f t="shared" si="4"/>
         <v>4</v>
       </c>
-      <c r="H19" s="16">
+      <c r="H19" s="14">
         <f t="shared" si="4"/>
         <v>5</v>
       </c>
-      <c r="I19" s="17">
+      <c r="I19" s="15">
         <f t="shared" si="4"/>
         <v>2</v>
       </c>
-      <c r="J19" s="17">
+      <c r="J19" s="15">
         <f t="shared" si="4"/>
         <v>3</v>
       </c>
-      <c r="K19" s="17">
+      <c r="K19" s="15">
         <f t="shared" si="4"/>
         <v>3</v>
       </c>
-      <c r="L19" s="18"/>
-      <c r="M19" s="11">
-        <v>1</v>
-      </c>
-      <c r="N19" s="35">
+      <c r="L19" s="16"/>
+      <c r="M19" s="9">
+        <v>1</v>
+      </c>
+      <c r="N19" s="30">
         <v>3.33</v>
       </c>
-      <c r="O19" s="42">
+      <c r="O19" s="37">
         <v>3</v>
       </c>
     </row>
     <row r="20" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A20" s="8" t="s">
-        <v>19</v>
-      </c>
-      <c r="B20" s="9" t="s">
-        <v>13</v>
-      </c>
-      <c r="C20" s="9">
+      <c r="A20" s="6" t="s">
+        <v>25</v>
+      </c>
+      <c r="B20" s="44" t="s">
+        <v>11</v>
+      </c>
+      <c r="C20" s="7">
         <v>7</v>
       </c>
-      <c r="D20" s="9">
+      <c r="D20" s="7">
         <v>7</v>
       </c>
-      <c r="E20" s="9">
+      <c r="E20" s="7">
         <v>7</v>
       </c>
-      <c r="F20" s="9">
-        <v>4</v>
-      </c>
-      <c r="G20" s="9">
+      <c r="F20" s="7">
+        <v>4</v>
+      </c>
+      <c r="G20" s="7">
         <v>7</v>
       </c>
-      <c r="H20" s="9">
+      <c r="H20" s="7">
         <v>7</v>
       </c>
-      <c r="I20" s="9">
-        <v>4</v>
-      </c>
-      <c r="J20" s="9">
-        <v>6</v>
-      </c>
-      <c r="K20" s="9">
+      <c r="I20" s="7">
+        <v>4</v>
+      </c>
+      <c r="J20" s="7">
+        <v>6</v>
+      </c>
+      <c r="K20" s="7">
         <v>8</v>
       </c>
-      <c r="L20" s="10"/>
-      <c r="M20" s="11"/>
-      <c r="N20" s="35"/>
-      <c r="O20" s="42"/>
+      <c r="L20" s="8"/>
+      <c r="M20" s="9"/>
+      <c r="N20" s="30"/>
+      <c r="O20" s="37"/>
     </row>
     <row r="21" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A21" s="12"/>
-      <c r="B21" s="13" t="s">
-        <v>7</v>
-      </c>
-      <c r="C21" s="13">
-        <v>2</v>
-      </c>
-      <c r="D21" s="13">
-        <v>2</v>
-      </c>
-      <c r="E21" s="13">
-        <v>2</v>
-      </c>
-      <c r="F21" s="13">
-        <v>1</v>
-      </c>
-      <c r="G21" s="13">
-        <v>2</v>
-      </c>
-      <c r="H21" s="13">
-        <v>2</v>
-      </c>
-      <c r="I21" s="13">
-        <v>2</v>
-      </c>
-      <c r="J21" s="13">
-        <v>2</v>
-      </c>
-      <c r="K21" s="13">
-        <v>2</v>
-      </c>
-      <c r="L21" s="14">
+      <c r="A21" s="10"/>
+      <c r="B21" s="45" t="s">
+        <v>6</v>
+      </c>
+      <c r="C21" s="11">
+        <v>2</v>
+      </c>
+      <c r="D21" s="11">
+        <v>2</v>
+      </c>
+      <c r="E21" s="11">
+        <v>2</v>
+      </c>
+      <c r="F21" s="11">
+        <v>1</v>
+      </c>
+      <c r="G21" s="11">
+        <v>2</v>
+      </c>
+      <c r="H21" s="11">
+        <v>2</v>
+      </c>
+      <c r="I21" s="11">
+        <v>2</v>
+      </c>
+      <c r="J21" s="11">
+        <v>2</v>
+      </c>
+      <c r="K21" s="11">
+        <v>2</v>
+      </c>
+      <c r="L21" s="12">
         <f>SUM(C21:K21)</f>
         <v>17</v>
       </c>
-      <c r="M21" s="11"/>
-      <c r="N21" s="35"/>
-      <c r="O21" s="42"/>
+      <c r="M21" s="9"/>
+      <c r="N21" s="30"/>
+      <c r="O21" s="37"/>
     </row>
     <row r="22" spans="1:15" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A22" s="15"/>
-      <c r="B22" s="16" t="s">
+      <c r="A22" s="13"/>
+      <c r="B22" s="46" t="s">
+        <v>12</v>
+      </c>
+      <c r="C22" s="14">
+        <f>C20-C21</f>
+        <v>5</v>
+      </c>
+      <c r="D22" s="14">
+        <f t="shared" ref="D22:K22" si="5">D20-D21</f>
+        <v>5</v>
+      </c>
+      <c r="E22" s="14">
+        <f t="shared" si="5"/>
+        <v>5</v>
+      </c>
+      <c r="F22" s="14">
+        <f t="shared" si="5"/>
+        <v>3</v>
+      </c>
+      <c r="G22" s="14">
+        <f t="shared" si="5"/>
+        <v>5</v>
+      </c>
+      <c r="H22" s="14">
+        <f t="shared" si="5"/>
+        <v>5</v>
+      </c>
+      <c r="I22" s="15">
+        <f t="shared" si="5"/>
+        <v>2</v>
+      </c>
+      <c r="J22" s="14">
+        <f t="shared" si="5"/>
+        <v>4</v>
+      </c>
+      <c r="K22" s="14">
+        <f t="shared" si="5"/>
+        <v>6</v>
+      </c>
+      <c r="L22" s="16"/>
+      <c r="M22" s="17">
+        <v>0</v>
+      </c>
+      <c r="N22" s="31">
+        <v>0</v>
+      </c>
+      <c r="O22" s="38"/>
+    </row>
+    <row r="23" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A23" s="18"/>
+      <c r="B23" s="18"/>
+      <c r="C23" s="18"/>
+      <c r="D23" s="18"/>
+      <c r="E23" s="18"/>
+      <c r="F23" s="18"/>
+      <c r="G23" s="18"/>
+      <c r="H23" s="18"/>
+      <c r="I23" s="18"/>
+      <c r="J23" s="18"/>
+      <c r="K23" s="18"/>
+      <c r="L23" s="18"/>
+      <c r="M23" s="19"/>
+      <c r="N23" s="32"/>
+      <c r="O23" s="39"/>
+    </row>
+    <row r="24" spans="1:15" s="51" customFormat="1" ht="12" x14ac:dyDescent="0.2">
+      <c r="A24" s="47"/>
+      <c r="B24" s="47"/>
+      <c r="C24" s="47" t="s">
+        <v>7</v>
+      </c>
+      <c r="D24" s="47" t="s">
+        <v>13</v>
+      </c>
+      <c r="E24" s="47" t="s">
+        <v>13</v>
+      </c>
+      <c r="F24" s="47" t="s">
         <v>14</v>
       </c>
-      <c r="C22" s="16">
-        <f>C20-C21</f>
-        <v>5</v>
-      </c>
-      <c r="D22" s="16">
-        <f t="shared" ref="D22:K22" si="5">D20-D21</f>
-        <v>5</v>
-      </c>
-      <c r="E22" s="16">
-        <f t="shared" si="5"/>
-        <v>5</v>
-      </c>
-      <c r="F22" s="16">
-        <f t="shared" si="5"/>
-        <v>3</v>
-      </c>
-      <c r="G22" s="16">
-        <f t="shared" si="5"/>
-        <v>5</v>
-      </c>
-      <c r="H22" s="16">
-        <f t="shared" si="5"/>
-        <v>5</v>
-      </c>
-      <c r="I22" s="17">
-        <f t="shared" si="5"/>
-        <v>2</v>
-      </c>
-      <c r="J22" s="16">
-        <f t="shared" si="5"/>
-        <v>4</v>
-      </c>
-      <c r="K22" s="16">
-        <f t="shared" si="5"/>
-        <v>6</v>
-      </c>
-      <c r="L22" s="18"/>
-      <c r="M22" s="19">
-        <v>0</v>
-      </c>
-      <c r="N22" s="36">
-        <v>0</v>
-      </c>
-      <c r="O22" s="43"/>
-    </row>
-    <row r="23" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A23" s="20"/>
-      <c r="B23" s="20"/>
-      <c r="C23" s="20"/>
-      <c r="D23" s="20"/>
-      <c r="E23" s="20"/>
-      <c r="F23" s="20"/>
-      <c r="G23" s="20"/>
-      <c r="H23" s="20"/>
-      <c r="I23" s="20"/>
-      <c r="J23" s="20"/>
-      <c r="K23" s="20"/>
-      <c r="L23" s="20"/>
-      <c r="M23" s="21"/>
-      <c r="N23" s="37"/>
-      <c r="O23" s="44"/>
-    </row>
-    <row r="24" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A24" s="20"/>
-      <c r="B24" s="20"/>
-      <c r="C24" s="20" t="s">
+      <c r="G24" s="47" t="s">
+        <v>15</v>
+      </c>
+      <c r="H24" s="47" t="s">
+        <v>16</v>
+      </c>
+      <c r="I24" s="47" t="s">
         <v>8</v>
       </c>
-      <c r="D24" s="20" t="s">
-        <v>20</v>
-      </c>
-      <c r="E24" s="20" t="s">
-        <v>20</v>
-      </c>
-      <c r="F24" s="20" t="s">
-        <v>21</v>
-      </c>
-      <c r="G24" s="20" t="s">
-        <v>22</v>
-      </c>
-      <c r="H24" s="20" t="s">
-        <v>23</v>
-      </c>
-      <c r="I24" s="20" t="s">
-        <v>9</v>
-      </c>
-      <c r="J24" s="20" t="s">
-        <v>8</v>
-      </c>
-      <c r="K24" s="20" t="s">
-        <v>24</v>
-      </c>
-      <c r="L24" s="20"/>
-      <c r="M24" s="21"/>
-      <c r="N24" s="37">
+      <c r="J24" s="47" t="s">
+        <v>7</v>
+      </c>
+      <c r="K24" s="47" t="s">
+        <v>17</v>
+      </c>
+      <c r="L24" s="47"/>
+      <c r="M24" s="48"/>
+      <c r="N24" s="49">
         <f>SUM(N7:N23)</f>
         <v>26.65</v>
       </c>
-      <c r="O24" s="44">
+      <c r="O24" s="50">
         <f>SUM(O7:O23)</f>
         <v>25</v>
       </c>
     </row>
-    <row r="25" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A25" s="20"/>
-      <c r="B25" s="20"/>
-      <c r="C25" s="20"/>
-      <c r="D25" s="20"/>
-      <c r="E25" s="20"/>
-      <c r="F25" s="20" t="s">
-        <v>10</v>
-      </c>
-      <c r="G25" s="20"/>
-      <c r="H25" s="20"/>
-      <c r="I25" s="20"/>
-      <c r="J25" s="20" t="s">
-        <v>25</v>
-      </c>
-      <c r="K25" s="20"/>
-      <c r="L25" s="20"/>
-      <c r="M25" s="21"/>
-      <c r="N25" s="37"/>
-      <c r="O25" s="37"/>
+    <row r="25" spans="1:15" s="51" customFormat="1" ht="12" x14ac:dyDescent="0.2">
+      <c r="A25" s="47"/>
+      <c r="B25" s="47"/>
+      <c r="C25" s="47"/>
+      <c r="D25" s="47"/>
+      <c r="E25" s="47"/>
+      <c r="F25" s="47" t="s">
+        <v>9</v>
+      </c>
+      <c r="G25" s="47"/>
+      <c r="H25" s="47"/>
+      <c r="I25" s="47"/>
+      <c r="J25" s="47" t="s">
+        <v>18</v>
+      </c>
+      <c r="K25" s="47"/>
+      <c r="L25" s="47"/>
+      <c r="M25" s="48"/>
+      <c r="N25" s="49"/>
+      <c r="O25" s="49"/>
     </row>
   </sheetData>
-  <mergeCells count="1">
+  <mergeCells count="2">
     <mergeCell ref="A1:L1"/>
+    <mergeCell ref="L2:L4"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="landscape" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>